<commit_message>
Add advanced Excel practice files
</commit_message>
<xml_diff>
--- a/5 Advance Excel in Data Analysis/11 DSUM List Function in Excel.xlsx
+++ b/5 Advance Excel in Data Analysis/11 DSUM List Function in Excel.xlsx
@@ -677,12 +677,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="13" formatCode="0%"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -723,6 +717,12 @@
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -737,29 +737,29 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6234B9DF-E4C7-43FF-88E0-E67086499402}" name="Table1" displayName="Table1" ref="A1:T51" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6234B9DF-E4C7-43FF-88E0-E67086499402}" name="Table1" displayName="Table1" ref="A1:T51" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
   <autoFilter ref="A1:T51" xr:uid="{6234B9DF-E4C7-43FF-88E0-E67086499402}"/>
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{8FB86759-7F89-445C-8B28-1DC1BAE2F11C}" name="Order_ID" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{4577A636-4DC6-4F08-B474-BA4AC00B719F}" name="Order_Date" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{4E4FCFBC-8749-484B-94EE-6B745D6AAD6E}" name="Customer_ID" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{59781B09-ABBC-4323-A02B-0D9D60C09D4C}" name="Customer_Name" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{28BCE014-EEFE-43A6-A1E5-9820A766CB3C}" name="Product_ID" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{F41E2C8F-4850-456E-9CAE-76AB8FF50311}" name="Product" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{8E1E79D3-581A-4A50-86A4-C7D759AF98FE}" name="Category" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{45D19338-8DBB-4E7F-B3E0-4EEAAFC6737D}" name="Country" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{DC311C0C-9879-47D4-8766-19ADAE51E090}" name="State" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{DEF6A1B8-A55E-42CA-A861-FB970154675C}" name="City" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{5C9EB120-74B4-4EC1-A0F0-B3DDB705D657}" name="Quantity" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{714ACD21-AE66-4A4D-A0AF-C6C5B770ADD3}" name="Unit_Price" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{B777B388-6B18-4C6D-B902-9F8B03AE93F5}" name="Discount" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{B9EAD4B9-0123-4B4B-82D5-F6B81C47A5B2}" name="Sales" dataDxfId="8"/>
-    <tableColumn id="15" xr3:uid="{0E3FF99E-C4EA-42CC-952C-29151D0F8168}" name="Cost" dataDxfId="7"/>
-    <tableColumn id="16" xr3:uid="{D7E79EC1-2347-435B-8059-2914BFDDE50E}" name="Profit" dataDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{14FA42A8-58DB-47BD-9ABF-9750F4E06A52}" name="Customer_Rating" dataDxfId="5"/>
-    <tableColumn id="18" xr3:uid="{934BD402-1DC1-45C9-80DB-64B839815CE6}" name="Payment_Method" dataDxfId="4"/>
-    <tableColumn id="19" xr3:uid="{D24EB1EF-DB13-47CF-BF2C-B738654F4578}" name="Sales_Channel" dataDxfId="3"/>
-    <tableColumn id="20" xr3:uid="{D1C15B87-9956-4AC5-98DC-1916D0BF4002}" name="Order_Status" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{8FB86759-7F89-445C-8B28-1DC1BAE2F11C}" name="Order_ID" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{4577A636-4DC6-4F08-B474-BA4AC00B719F}" name="Order_Date" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{4E4FCFBC-8749-484B-94EE-6B745D6AAD6E}" name="Customer_ID" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{59781B09-ABBC-4323-A02B-0D9D60C09D4C}" name="Customer_Name" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{28BCE014-EEFE-43A6-A1E5-9820A766CB3C}" name="Product_ID" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{F41E2C8F-4850-456E-9CAE-76AB8FF50311}" name="Product" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{8E1E79D3-581A-4A50-86A4-C7D759AF98FE}" name="Category" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{45D19338-8DBB-4E7F-B3E0-4EEAAFC6737D}" name="Country" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{DC311C0C-9879-47D4-8766-19ADAE51E090}" name="State" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{DEF6A1B8-A55E-42CA-A861-FB970154675C}" name="City" dataDxfId="10"/>
+    <tableColumn id="11" xr3:uid="{5C9EB120-74B4-4EC1-A0F0-B3DDB705D657}" name="Quantity" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{714ACD21-AE66-4A4D-A0AF-C6C5B770ADD3}" name="Unit_Price" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{B777B388-6B18-4C6D-B902-9F8B03AE93F5}" name="Discount" dataDxfId="7"/>
+    <tableColumn id="14" xr3:uid="{B9EAD4B9-0123-4B4B-82D5-F6B81C47A5B2}" name="Sales" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{0E3FF99E-C4EA-42CC-952C-29151D0F8168}" name="Cost" dataDxfId="5"/>
+    <tableColumn id="16" xr3:uid="{D7E79EC1-2347-435B-8059-2914BFDDE50E}" name="Profit" dataDxfId="4"/>
+    <tableColumn id="17" xr3:uid="{14FA42A8-58DB-47BD-9ABF-9750F4E06A52}" name="Customer_Rating" dataDxfId="3"/>
+    <tableColumn id="18" xr3:uid="{934BD402-1DC1-45C9-80DB-64B839815CE6}" name="Payment_Method" dataDxfId="2"/>
+    <tableColumn id="19" xr3:uid="{D24EB1EF-DB13-47CF-BF2C-B738654F4578}" name="Sales_Channel" dataDxfId="1"/>
+    <tableColumn id="20" xr3:uid="{D1C15B87-9956-4AC5-98DC-1916D0BF4002}" name="Order_Status" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>